<commit_message>
update labels Fixes #10
</commit_message>
<xml_diff>
--- a/data/codebooks/codebook_columns.xlsx
+++ b/data/codebooks/codebook_columns.xlsx
@@ -577,7 +577,7 @@
     <t>Strukturanpassung_Folge</t>
   </si>
   <si>
-    <t>[03.09] Structural adjustment</t>
+    <t/>
   </si>
   <si>
     <t>[03.10.01] Folgen - Wer hat geprüft?</t>
@@ -673,7 +673,7 @@
     <t>Ende_vs_Pause</t>
   </si>
   <si>
-    <t>[03.13.01] Suspension or termination of session</t>
+    <t>[03.13.01] Temporary suspension of session</t>
   </si>
   <si>
     <t>[03.13.02] Folgen - Wie lange wurde pausiert?</t>
@@ -1031,7 +1031,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1067,6 +1067,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -1380,16 +1383,16 @@
   <dimension ref="A1:G118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="13" width="73.29071428571429" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="13" width="9.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="13" width="42.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="13" width="53.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="13" width="53.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="14" width="73.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="14" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="14" width="42.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="14" width="53.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="14" width="53.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1412,7 +1415,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
@@ -1429,7 +1432,7 @@
       </c>
       <c r="G2" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
@@ -1446,7 +1449,7 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
@@ -1463,7 +1466,7 @@
       </c>
       <c r="G4" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
@@ -1480,7 +1483,7 @@
       </c>
       <c r="G5" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="4" t="s">
         <v>15</v>
       </c>
@@ -1497,7 +1500,7 @@
       </c>
       <c r="G6" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="4" t="s">
         <v>17</v>
       </c>
@@ -1514,7 +1517,7 @@
       </c>
       <c r="G7" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="4" t="s">
         <v>19</v>
       </c>
@@ -1531,7 +1534,7 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="4" t="s">
         <v>21</v>
       </c>
@@ -1548,7 +1551,7 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="4" t="s">
         <v>23</v>
       </c>
@@ -1565,7 +1568,7 @@
       </c>
       <c r="G10" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="4" t="s">
         <v>25</v>
       </c>
@@ -1582,7 +1585,7 @@
       </c>
       <c r="G11" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="4" t="s">
         <v>27</v>
       </c>
@@ -1599,7 +1602,7 @@
       </c>
       <c r="G12" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="4" t="s">
         <v>29</v>
       </c>
@@ -1616,7 +1619,7 @@
       </c>
       <c r="G13" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="4" t="s">
         <v>31</v>
       </c>
@@ -1633,7 +1636,7 @@
       </c>
       <c r="G14" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="4" t="s">
         <v>33</v>
       </c>
@@ -1650,7 +1653,7 @@
       </c>
       <c r="G15" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="4" t="s">
         <v>35</v>
       </c>
@@ -1667,7 +1670,7 @@
       </c>
       <c r="G16" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="4" t="s">
         <v>37</v>
       </c>
@@ -1684,7 +1687,7 @@
       </c>
       <c r="G17" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="4" t="s">
         <v>39</v>
       </c>
@@ -1703,7 +1706,7 @@
         <v>40</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="4" t="s">
         <v>41</v>
       </c>
@@ -1720,7 +1723,7 @@
       </c>
       <c r="G19" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="4" t="s">
         <v>42</v>
       </c>
@@ -1737,7 +1740,7 @@
       </c>
       <c r="G20" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="4" t="s">
         <v>43</v>
       </c>
@@ -1754,7 +1757,7 @@
       </c>
       <c r="G21" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="4" t="s">
         <v>45</v>
       </c>
@@ -1771,7 +1774,7 @@
       </c>
       <c r="G22" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="4" t="s">
         <v>47</v>
       </c>
@@ -1788,7 +1791,7 @@
       </c>
       <c r="G23" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="4" t="s">
         <v>49</v>
       </c>
@@ -1805,7 +1808,7 @@
       </c>
       <c r="G24" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="4" t="s">
         <v>51</v>
       </c>
@@ -1822,7 +1825,7 @@
       </c>
       <c r="G25" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="4" t="s">
         <v>53</v>
       </c>
@@ -1839,7 +1842,7 @@
       </c>
       <c r="G26" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="4" t="s">
         <v>55</v>
       </c>
@@ -1856,7 +1859,7 @@
       </c>
       <c r="G27" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="4" t="s">
         <v>57</v>
       </c>
@@ -1873,7 +1876,7 @@
       </c>
       <c r="G28" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="4" t="s">
         <v>59</v>
       </c>
@@ -1890,7 +1893,7 @@
       </c>
       <c r="G29" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="4" t="s">
         <v>61</v>
       </c>
@@ -1907,7 +1910,7 @@
       </c>
       <c r="G30" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="4" t="s">
         <v>63</v>
       </c>
@@ -1924,7 +1927,7 @@
       </c>
       <c r="G31" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="4" t="s">
         <v>65</v>
       </c>
@@ -1941,7 +1944,7 @@
       </c>
       <c r="G32" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="4" t="s">
         <v>67</v>
       </c>
@@ -1958,7 +1961,7 @@
       </c>
       <c r="G33" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="4" t="s">
         <v>69</v>
       </c>
@@ -1975,7 +1978,7 @@
       </c>
       <c r="G34" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="4" t="s">
         <v>71</v>
       </c>
@@ -2616,7 +2619,7 @@
       </c>
       <c r="G69" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
       <c r="A70" s="9" t="s">
         <v>164</v>
       </c>
@@ -2633,7 +2636,7 @@
       </c>
       <c r="G70" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
       <c r="A71" s="9" t="s">
         <v>166</v>
       </c>
@@ -2654,7 +2657,7 @@
         <v>169</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
       <c r="A72" s="9" t="s">
         <v>170</v>
       </c>
@@ -2675,7 +2678,7 @@
         <v>173</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
       <c r="A73" s="9" t="s">
         <v>174</v>
       </c>
@@ -2692,7 +2695,7 @@
       </c>
       <c r="G73" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
       <c r="A74" s="9" t="s">
         <v>176</v>
       </c>
@@ -2713,7 +2716,7 @@
         <v>179</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
       <c r="A75" s="9" t="s">
         <v>180</v>
       </c>
@@ -2730,7 +2733,7 @@
       </c>
       <c r="G75" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
       <c r="A76" s="9" t="s">
         <v>182</v>
       </c>
@@ -2747,7 +2750,7 @@
       </c>
       <c r="G76" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
       <c r="A77" s="9" t="s">
         <v>184</v>
       </c>
@@ -2764,11 +2767,11 @@
       <c r="F77" s="11">
         <f>_xlfn.CONCAT(B77, , " ", D77)</f>
       </c>
-      <c r="G77" s="9" t="s">
+      <c r="G77" s="13" t="s">
         <v>187</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
       <c r="A78" s="9" t="s">
         <v>188</v>
       </c>
@@ -2789,7 +2792,7 @@
         <v>191</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
       <c r="A79" s="9" t="s">
         <v>192</v>
       </c>
@@ -2810,7 +2813,7 @@
         <v>195</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
       <c r="A80" s="9" t="s">
         <v>196</v>
       </c>
@@ -2831,7 +2834,7 @@
         <v>199</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
       <c r="A81" s="9" t="s">
         <v>200</v>
       </c>
@@ -2848,7 +2851,7 @@
       </c>
       <c r="G81" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
       <c r="A82" s="9" t="s">
         <v>202</v>
       </c>
@@ -2865,7 +2868,7 @@
       </c>
       <c r="G82" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
       <c r="A83" s="9" t="s">
         <v>204</v>
       </c>
@@ -2886,7 +2889,7 @@
         <v>206</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
       <c r="A84" s="9" t="s">
         <v>207</v>
       </c>
@@ -2905,7 +2908,7 @@
       </c>
       <c r="G84" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
       <c r="A85" s="9" t="s">
         <v>210</v>
       </c>
@@ -2922,7 +2925,7 @@
       </c>
       <c r="G85" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
       <c r="A86" s="9" t="s">
         <v>212</v>
       </c>
@@ -2943,7 +2946,7 @@
         <v>215</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
       <c r="A87" s="9" t="s">
         <v>216</v>
       </c>
@@ -2964,7 +2967,7 @@
         <v>219</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
       <c r="A88" s="9" t="s">
         <v>220</v>
       </c>
@@ -2981,7 +2984,7 @@
       </c>
       <c r="G88" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
       <c r="A89" s="9" t="s">
         <v>222</v>
       </c>
@@ -3002,7 +3005,7 @@
         <v>225</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
       <c r="A90" s="9" t="s">
         <v>226</v>
       </c>
@@ -3023,7 +3026,7 @@
         <v>229</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
       <c r="A91" s="9" t="s">
         <v>230</v>
       </c>
@@ -3042,7 +3045,7 @@
       </c>
       <c r="G91" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
       <c r="A92" s="9" t="s">
         <v>233</v>
       </c>
@@ -3063,7 +3066,7 @@
         <v>236</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
       <c r="A93" s="9" t="s">
         <v>237</v>
       </c>
@@ -3080,7 +3083,7 @@
       </c>
       <c r="G93" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
       <c r="A94" s="9" t="s">
         <v>239</v>
       </c>
@@ -3097,7 +3100,7 @@
       </c>
       <c r="G94" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
       <c r="A95" s="9" t="s">
         <v>241</v>
       </c>
@@ -3114,7 +3117,7 @@
       </c>
       <c r="G95" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
       <c r="A96" s="9" t="s">
         <v>243</v>
       </c>
@@ -3135,7 +3138,7 @@
         <v>246</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
       <c r="A97" s="9" t="s">
         <v>247</v>
       </c>
@@ -3152,7 +3155,7 @@
       </c>
       <c r="G97" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
       <c r="A98" s="9" t="s">
         <v>249</v>
       </c>
@@ -3169,7 +3172,7 @@
       </c>
       <c r="G98" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
       <c r="A99" s="9" t="s">
         <v>251</v>
       </c>
@@ -3186,7 +3189,7 @@
       </c>
       <c r="G99" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
       <c r="A100" s="9" t="s">
         <v>253</v>
       </c>
@@ -3203,7 +3206,7 @@
       </c>
       <c r="G100" s="9"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
       <c r="A101" s="9" t="s">
         <v>255</v>
       </c>
@@ -3224,7 +3227,7 @@
         <v>257</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
       <c r="A102" s="9" t="s">
         <v>258</v>
       </c>
@@ -3245,7 +3248,7 @@
         <v>260</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
       <c r="A103" s="9" t="s">
         <v>261</v>
       </c>

</xml_diff>

<commit_message>
update labels Fixes #10 introduce upset plot Fixes #11
</commit_message>
<xml_diff>
--- a/data/codebooks/codebook_columns.xlsx
+++ b/data/codebooks/codebook_columns.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="301">
   <si>
     <t>col_clean</t>
   </si>
@@ -577,9 +577,6 @@
     <t>Strukturanpassung_Folge</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>[03.10.01] Folgen - Wer hat geprüft?</t>
   </si>
   <si>
@@ -832,7 +829,10 @@
     <t>[05.06]</t>
   </si>
   <si>
-    <t>[05.06] Setting</t>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>[05.06] Location</t>
   </si>
   <si>
     <t xml:space="preserve">[05.07] Rahmenbedingungen - Welche motorische Hauptform dominierte die Bewegungseinheit? </t>
@@ -1031,7 +1031,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1067,9 +1067,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -1383,13 +1380,13 @@
   <dimension ref="A1:G118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="14" width="73.29071428571429" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="14" width="9.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="42.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="14" width="53.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="14" width="53.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="13" width="73.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="13" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="13" width="42.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="13" width="53.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="13" width="53.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -2767,83 +2764,81 @@
       <c r="F77" s="11">
         <f>_xlfn.CONCAT(B77, , " ", D77)</f>
       </c>
-      <c r="G77" s="13" t="s">
-        <v>187</v>
-      </c>
+      <c r="G77" s="9"/>
     </row>
     <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
       <c r="A78" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="B78" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="B78" s="9" t="s">
+      <c r="C78" s="10">
+        <v>1</v>
+      </c>
+      <c r="D78" s="9" t="s">
         <v>189</v>
-      </c>
-      <c r="C78" s="10">
-        <v>1</v>
-      </c>
-      <c r="D78" s="9" t="s">
-        <v>190</v>
       </c>
       <c r="E78" s="9"/>
       <c r="F78" s="11">
         <f>_xlfn.CONCAT(B78, , " ", D78)</f>
       </c>
       <c r="G78" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
       <c r="A79" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="B79" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="B79" s="9" t="s">
+      <c r="C79" s="10">
+        <v>1</v>
+      </c>
+      <c r="D79" s="9" t="s">
         <v>193</v>
-      </c>
-      <c r="C79" s="10">
-        <v>1</v>
-      </c>
-      <c r="D79" s="9" t="s">
-        <v>194</v>
       </c>
       <c r="E79" s="9"/>
       <c r="F79" s="11">
         <f>_xlfn.CONCAT(B79, , " ", D79)</f>
       </c>
       <c r="G79" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
       <c r="A80" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B80" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="B80" s="9" t="s">
+      <c r="C80" s="10">
+        <v>1</v>
+      </c>
+      <c r="D80" s="9" t="s">
         <v>197</v>
-      </c>
-      <c r="C80" s="10">
-        <v>1</v>
-      </c>
-      <c r="D80" s="9" t="s">
-        <v>198</v>
       </c>
       <c r="E80" s="9"/>
       <c r="F80" s="11">
         <f>_xlfn.CONCAT(B80, , " ", D80)</f>
       </c>
       <c r="G80" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
       <c r="A81" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B81" s="9"/>
       <c r="C81" s="10">
         <v>4</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E81" s="9"/>
       <c r="F81" s="11">
@@ -2853,14 +2848,14 @@
     </row>
     <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
       <c r="A82" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B82" s="9"/>
       <c r="C82" s="10">
         <v>1</v>
       </c>
       <c r="D82" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E82" s="9"/>
       <c r="F82" s="11">
@@ -2870,37 +2865,37 @@
     </row>
     <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
       <c r="A83" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="B83" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="B83" s="9" t="s">
-        <v>205</v>
-      </c>
       <c r="C83" s="10">
         <v>1</v>
       </c>
       <c r="D83" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E83" s="9"/>
       <c r="F83" s="11">
         <f>_xlfn.CONCAT(B83, , " ", D83)</f>
       </c>
       <c r="G83" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
       <c r="A84" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="B84" s="9" t="s">
         <v>207</v>
-      </c>
-      <c r="B84" s="9" t="s">
-        <v>208</v>
       </c>
       <c r="C84" s="10">
         <v>6</v>
       </c>
       <c r="D84" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E84" s="9"/>
       <c r="F84" s="11">
@@ -2910,14 +2905,14 @@
     </row>
     <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
       <c r="A85" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B85" s="9"/>
       <c r="C85" s="10">
         <v>1</v>
       </c>
       <c r="D85" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E85" s="9"/>
       <c r="F85" s="11">
@@ -2927,56 +2922,56 @@
     </row>
     <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
       <c r="A86" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="B86" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="B86" s="9" t="s">
+      <c r="C86" s="10">
+        <v>1</v>
+      </c>
+      <c r="D86" s="9" t="s">
         <v>213</v>
-      </c>
-      <c r="C86" s="10">
-        <v>1</v>
-      </c>
-      <c r="D86" s="9" t="s">
-        <v>214</v>
       </c>
       <c r="E86" s="9"/>
       <c r="F86" s="11">
         <f>_xlfn.CONCAT(B86, , " ", D86)</f>
       </c>
       <c r="G86" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
       <c r="A87" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="B87" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="B87" s="9" t="s">
+      <c r="C87" s="10">
+        <v>1</v>
+      </c>
+      <c r="D87" s="9" t="s">
         <v>217</v>
-      </c>
-      <c r="C87" s="10">
-        <v>1</v>
-      </c>
-      <c r="D87" s="9" t="s">
-        <v>218</v>
       </c>
       <c r="E87" s="9"/>
       <c r="F87" s="11">
         <f>_xlfn.CONCAT(B87, , " ", D87)</f>
       </c>
       <c r="G87" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
       <c r="A88" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B88" s="9"/>
       <c r="C88" s="10">
         <v>1</v>
       </c>
       <c r="D88" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E88" s="9"/>
       <c r="F88" s="11">
@@ -2986,58 +2981,58 @@
     </row>
     <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
       <c r="A89" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="B89" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="B89" s="9" t="s">
+      <c r="C89" s="10">
+        <v>1</v>
+      </c>
+      <c r="D89" s="9" t="s">
         <v>223</v>
-      </c>
-      <c r="C89" s="10">
-        <v>1</v>
-      </c>
-      <c r="D89" s="9" t="s">
-        <v>224</v>
       </c>
       <c r="E89" s="9"/>
       <c r="F89" s="11">
         <f>_xlfn.CONCAT(B89, , " ", D89)</f>
       </c>
       <c r="G89" s="9" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
       <c r="A90" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="B90" s="9" t="s">
         <v>226</v>
-      </c>
-      <c r="B90" s="9" t="s">
-        <v>227</v>
       </c>
       <c r="C90" s="10">
         <v>9</v>
       </c>
       <c r="D90" s="9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E90" s="9"/>
       <c r="F90" s="11">
         <f>_xlfn.CONCAT(B90, , " ", D90)</f>
       </c>
       <c r="G90" s="9" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
       <c r="A91" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="B91" s="9" t="s">
         <v>230</v>
-      </c>
-      <c r="B91" s="9" t="s">
-        <v>231</v>
       </c>
       <c r="C91" s="10">
         <v>3</v>
       </c>
       <c r="D91" s="9" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E91" s="9"/>
       <c r="F91" s="11">
@@ -3047,35 +3042,35 @@
     </row>
     <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
       <c r="A92" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B92" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="B92" s="9" t="s">
+      <c r="C92" s="10">
+        <v>1</v>
+      </c>
+      <c r="D92" s="9" t="s">
         <v>234</v>
-      </c>
-      <c r="C92" s="10">
-        <v>1</v>
-      </c>
-      <c r="D92" s="9" t="s">
-        <v>235</v>
       </c>
       <c r="E92" s="9"/>
       <c r="F92" s="11">
         <f>_xlfn.CONCAT(B92, , " ", D92)</f>
       </c>
       <c r="G92" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
       <c r="A93" s="9" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B93" s="9"/>
       <c r="C93" s="10">
         <v>2</v>
       </c>
       <c r="D93" s="9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E93" s="9"/>
       <c r="F93" s="11">
@@ -3085,14 +3080,14 @@
     </row>
     <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
       <c r="A94" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B94" s="9"/>
       <c r="C94" s="10">
         <v>1</v>
       </c>
       <c r="D94" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E94" s="9"/>
       <c r="F94" s="11">
@@ -3102,14 +3097,14 @@
     </row>
     <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
       <c r="A95" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B95" s="9"/>
       <c r="C95" s="10">
         <v>1</v>
       </c>
       <c r="D95" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E95" s="9"/>
       <c r="F95" s="11">
@@ -3119,35 +3114,35 @@
     </row>
     <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
       <c r="A96" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="B96" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="B96" s="9" t="s">
+      <c r="C96" s="10">
+        <v>1</v>
+      </c>
+      <c r="D96" s="9" t="s">
         <v>244</v>
-      </c>
-      <c r="C96" s="10">
-        <v>1</v>
-      </c>
-      <c r="D96" s="9" t="s">
-        <v>245</v>
       </c>
       <c r="E96" s="9"/>
       <c r="F96" s="11">
         <f>_xlfn.CONCAT(B96, , " ", D96)</f>
       </c>
       <c r="G96" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
       <c r="A97" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B97" s="9"/>
       <c r="C97" s="10">
         <v>3</v>
       </c>
       <c r="D97" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E97" s="9"/>
       <c r="F97" s="11">
@@ -3157,14 +3152,14 @@
     </row>
     <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
       <c r="A98" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B98" s="9"/>
       <c r="C98" s="10">
         <v>1</v>
       </c>
       <c r="D98" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E98" s="9"/>
       <c r="F98" s="11">
@@ -3174,14 +3169,14 @@
     </row>
     <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
       <c r="A99" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B99" s="9"/>
       <c r="C99" s="10">
         <v>1</v>
       </c>
       <c r="D99" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E99" s="9"/>
       <c r="F99" s="11">
@@ -3191,14 +3186,14 @@
     </row>
     <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
       <c r="A100" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B100" s="9"/>
       <c r="C100" s="10">
         <v>1</v>
       </c>
       <c r="D100" s="9" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E100" s="9"/>
       <c r="F100" s="11">
@@ -3208,10 +3203,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
       <c r="A101" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="B101" s="9" t="s">
         <v>255</v>
-      </c>
-      <c r="B101" s="9" t="s">
-        <v>256</v>
       </c>
       <c r="C101" s="10">
         <v>1</v>
@@ -3224,15 +3219,15 @@
         <f>_xlfn.CONCAT(B101, , " ", D101)</f>
       </c>
       <c r="G101" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
       <c r="A102" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="B102" s="9" t="s">
         <v>258</v>
-      </c>
-      <c r="B102" s="9" t="s">
-        <v>259</v>
       </c>
       <c r="C102" s="10">
         <v>1</v>
@@ -3245,15 +3240,15 @@
         <f>_xlfn.CONCAT(B102, , " ", D102)</f>
       </c>
       <c r="G102" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
       <c r="A103" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="B103" s="9" t="s">
         <v>261</v>
-      </c>
-      <c r="B103" s="9" t="s">
-        <v>262</v>
       </c>
       <c r="C103" s="10">
         <v>1</v>
@@ -3266,15 +3261,15 @@
         <f>_xlfn.CONCAT(B103, , " ", D103)</f>
       </c>
       <c r="G103" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18">
       <c r="A104" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="B104" s="9" t="s">
         <v>264</v>
-      </c>
-      <c r="B104" s="9" t="s">
-        <v>265</v>
       </c>
       <c r="C104" s="10">
         <v>1</v>
@@ -3287,15 +3282,15 @@
         <f>_xlfn.CONCAT(B104, , " ", D104)</f>
       </c>
       <c r="G104" s="9" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18">
       <c r="A105" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="B105" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="B105" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="C105" s="10">
         <v>1</v>
@@ -3308,21 +3303,21 @@
         <f>_xlfn.CONCAT(B105, , " ", D105)</f>
       </c>
       <c r="G105" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18">
       <c r="A106" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="B106" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="B106" s="9" t="s">
+      <c r="C106" s="10">
+        <v>1</v>
+      </c>
+      <c r="D106" s="9" t="s">
         <v>271</v>
-      </c>
-      <c r="C106" s="10">
-        <v>1</v>
-      </c>
-      <c r="D106" s="9" t="s">
-        <v>32</v>
       </c>
       <c r="E106" s="9"/>
       <c r="F106" s="11">

</xml_diff>